<commit_message>
Cambio plantillas, reporte valorizado
</commit_message>
<xml_diff>
--- a/TomaInventarioWEB/Plantillas/Plantilla_Inventario.xlsx
+++ b/TomaInventarioWEB/Plantillas/Plantilla_Inventario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\User\Desktop\Documentos\TomaDeInventario - Web\TomaInventario-GitHub\TomaInventarioWEB\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{494FF686-9D03-4D01-B75D-476B32818CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C57FE10-B74D-4310-8C02-D9923DDDE821}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30720" yWindow="1320" windowWidth="26085" windowHeight="14160" tabRatio="983" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="983" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="18" r:id="rId1"/>
@@ -114,17 +114,17 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -432,32 +432,32 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
     </row>
   </sheetData>
   <dataConsolidate/>

</xml_diff>